<commit_message>
Add clickable cards with modals in Dashboard tab
</commit_message>
<xml_diff>
--- a/daily_dashboard1.xlsx
+++ b/daily_dashboard1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tonio\Documents\dashboard-industriel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E099DA23-C7B0-46F5-8AC6-285D058838E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{902E9788-C345-444D-B8C1-B71CBD2624A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KPI_Daily" sheetId="1" r:id="rId1"/>
@@ -196,10 +196,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -677,7 +683,7 @@
         <v>12</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -699,6 +705,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -814,7 +821,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
update Excel with new actions format, remove old versions
</commit_message>
<xml_diff>
--- a/daily_dashboard1.xlsx
+++ b/daily_dashboard1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tonio\Documents\dashboard-industriel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{902E9788-C345-444D-B8C1-B71CBD2624A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547D38F5-406A-402A-9972-8AFD11BDAB2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KPI_Daily" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="48">
   <si>
     <t>Date</t>
   </si>
@@ -138,58 +138,40 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Drehmaschine</t>
-  </si>
-  <si>
-    <t>Jörg B</t>
-  </si>
-  <si>
-    <t>Angebot holen und bestellen</t>
-  </si>
-  <si>
-    <t>20/02/2026</t>
-  </si>
-  <si>
-    <t>Überfällig</t>
-  </si>
-  <si>
-    <t>Cu-Glas Faser Verbindung</t>
-  </si>
-  <si>
-    <t>Teil bestellen, Hersteller kontaktieren</t>
-  </si>
-  <si>
-    <t>Dimos Reparatur</t>
-  </si>
-  <si>
-    <t>05/02/2026</t>
-  </si>
-  <si>
-    <t>Adrian</t>
-  </si>
-  <si>
-    <t>Warten auf das Angebot</t>
-  </si>
-  <si>
-    <t>13/02/2026</t>
-  </si>
-  <si>
-    <t>Neue Maschine</t>
-  </si>
-  <si>
-    <t>15/02/2026</t>
-  </si>
-  <si>
-    <t>Klaus M</t>
-  </si>
-  <si>
-    <t>Installation planen</t>
-  </si>
-  <si>
-    <t>01/03/2026</t>
-  </si>
-  <si>
-    <t>In Progress</t>
+    <t>Thema 1</t>
+  </si>
+  <si>
+    <t>Thema 2</t>
+  </si>
+  <si>
+    <t>Thema 3</t>
+  </si>
+  <si>
+    <t>Thema 4</t>
+  </si>
+  <si>
+    <t>Antonio</t>
+  </si>
+  <si>
+    <t>Aktion 1</t>
+  </si>
+  <si>
+    <t>Aktion 2</t>
+  </si>
+  <si>
+    <t>Aktion 3</t>
+  </si>
+  <si>
+    <t>Aktion 4</t>
+  </si>
+  <si>
+    <t>Not started</t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>Completed</t>
   </si>
 </sst>
 </file>
@@ -231,8 +213,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -712,7 +695,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="6" customWidth="1"/>
@@ -774,6 +757,17 @@
       </c>
       <c r="D4">
         <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>2026</v>
+      </c>
+      <c r="C5">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -878,7 +872,7 @@
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="41" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
   </cols>
@@ -913,17 +907,20 @@
       <c r="B2" t="s">
         <v>36</v>
       </c>
+      <c r="C2" s="1">
+        <v>46086</v>
+      </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" t="s">
-        <v>39</v>
+        <v>41</v>
+      </c>
+      <c r="F2" s="1">
+        <v>46091</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -931,19 +928,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>37</v>
+      </c>
+      <c r="C3" s="1">
+        <v>46087</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
         <v>42</v>
       </c>
-      <c r="F3" t="s">
-        <v>39</v>
+      <c r="F3" s="1">
+        <v>46088</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -951,22 +951,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="1">
+        <v>46088</v>
+      </c>
+      <c r="D4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" t="s">
         <v>43</v>
       </c>
-      <c r="C4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="F4" s="1">
+        <v>46093</v>
+      </c>
+      <c r="G4" t="s">
         <v>47</v>
-      </c>
-      <c r="G4" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,25 +974,31 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" t="s">
-        <v>49</v>
+        <v>39</v>
+      </c>
+      <c r="C5" s="1">
+        <v>46089</v>
       </c>
       <c r="D5" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>51</v>
-      </c>
-      <c r="F5" t="s">
-        <v>52</v>
+        <v>44</v>
+      </c>
+      <c r="F5" s="1">
+        <v>46094</v>
       </c>
       <c r="G5" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G35" xr:uid="{DD123BC6-4D6B-4A22-BFA4-7B9F5E305215}">
+      <formula1>"Not started,In progress,Completed"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>